<commit_message>
First run with reward saltation, but ran into some agenda issue.
</commit_message>
<xml_diff>
--- a/data/c_vs_random.xlsx
+++ b/data/c_vs_random.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -665,6 +665,17 @@
         <v>31.292</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="B22" t="n">
+        <v>95.8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>31.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
First set of reward saltation models, no breaktrought yet.
</commit_message>
<xml_diff>
--- a/data/c_vs_random.xlsx
+++ b/data/c_vs_random.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -676,6 +676,105 @@
         <v>31.13</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="B23" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="C23" t="n">
+        <v>31.436</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>90</v>
+      </c>
+      <c r="B24" t="n">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="C24" t="n">
+        <v>31.616</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>92</v>
+      </c>
+      <c r="B25" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="C25" t="n">
+        <v>31.663</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>94</v>
+      </c>
+      <c r="B26" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>31.487</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>96</v>
+      </c>
+      <c r="B27" t="n">
+        <v>93.7</v>
+      </c>
+      <c r="C27" t="n">
+        <v>31.388</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>98</v>
+      </c>
+      <c r="B28" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="C28" t="n">
+        <v>31.218</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="B29" t="n">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="C29" t="n">
+        <v>30.994</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>102</v>
+      </c>
+      <c r="B30" t="n">
+        <v>94</v>
+      </c>
+      <c r="C30" t="n">
+        <v>31.704</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>104</v>
+      </c>
+      <c r="B31" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="C31" t="n">
+        <v>31.437</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
First pass with proper reward saltation.
</commit_message>
<xml_diff>
--- a/data/c_vs_random.xlsx
+++ b/data/c_vs_random.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -775,6 +775,193 @@
         <v>31.437</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>106</v>
+      </c>
+      <c r="B32" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="C32" t="n">
+        <v>31.468</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="B33" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>31.255</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>110</v>
+      </c>
+      <c r="B34" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>31.522</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>112</v>
+      </c>
+      <c r="B35" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="C35" t="n">
+        <v>31.499</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>114</v>
+      </c>
+      <c r="B36" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="C36" t="n">
+        <v>31.698</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B37" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="C37" t="n">
+        <v>31.239</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B38" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="C38" t="n">
+        <v>31.558</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>120</v>
+      </c>
+      <c r="B39" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="C39" t="n">
+        <v>31.459</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>122</v>
+      </c>
+      <c r="B40" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="C40" t="n">
+        <v>31.498</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>124</v>
+      </c>
+      <c r="B41" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>31.728</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>126</v>
+      </c>
+      <c r="B42" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="C42" t="n">
+        <v>31.643</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>128</v>
+      </c>
+      <c r="B43" t="n">
+        <v>95.09999999999999</v>
+      </c>
+      <c r="C43" t="n">
+        <v>31.33</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>130</v>
+      </c>
+      <c r="B44" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="C44" t="n">
+        <v>31.637</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>132</v>
+      </c>
+      <c r="B45" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="C45" t="n">
+        <v>31.512</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>134</v>
+      </c>
+      <c r="B46" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="C46" t="n">
+        <v>31.437</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>136</v>
+      </c>
+      <c r="B47" t="n">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="C47" t="n">
+        <v>31.462</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>138</v>
+      </c>
+      <c r="B48" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="C48" t="n">
+        <v>31.583</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>